<commit_message>
Revert "Publication ans.fhir.fr.annuaire 1.2.0-snapshot-1"
This reverts commit 1be070afe1096ab3e54199d18c796b68d1cd5ba6.
</commit_message>
<xml_diff>
--- a/www/ig/fhir/annuaire/1.2.0-snapshot-1/CodeSystem-as-cs-organization-types.xlsx
+++ b/www/ig/fhir/annuaire/1.2.0-snapshot-1/CodeSystem-as-cs-organization-types.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.2.0-snapshot-2</t>
+    <t>1.2.0-snapshot-1</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-19T14:20:56+00:00</t>
+    <t>2026-06-16T14:13:23+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Revert "Publication ans.fhir.fr.annuaire 1.2.0-snapshot-1" (#62)
This reverts commit 1be070afe1096ab3e54199d18c796b68d1cd5ba6.
</commit_message>
<xml_diff>
--- a/www/ig/fhir/annuaire/1.2.0-snapshot-1/CodeSystem-as-cs-organization-types.xlsx
+++ b/www/ig/fhir/annuaire/1.2.0-snapshot-1/CodeSystem-as-cs-organization-types.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.2.0-snapshot-2</t>
+    <t>1.2.0-snapshot-1</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-19T14:20:56+00:00</t>
+    <t>2026-06-16T14:13:23+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>